<commit_message>
adds SE london ICB to the lookup list of focal ICBs
</commit_message>
<xml_diff>
--- a/data/project/focal_icbs.xlsx
+++ b/data/project/focal_icbs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nhs-my.sharepoint.com/personal/craig_parylo2_nhs_net/Documents/Documents/Projects/1199_core20plus5/data/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="11_F25DC773A252ABDACC10485B515949AE5BDE58F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C110B088-DF1E-4D3E-ACE7-9CB6DED8B408}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="11_F25DC773A252ABDACC10485B515949AE5BDE58F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7EFA22B-A835-4347-9BB9-82603B7B4B37}"/>
   <bookViews>
-    <workbookView xWindow="23070" yWindow="2490" windowWidth="12675" windowHeight="10770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19020" yWindow="0" windowWidth="19290" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="focal_icbs" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
   <si>
     <t>nhs_region</t>
   </si>
@@ -139,6 +139,12 @@
   </si>
   <si>
     <t>NHS Nottingham and Nottinghamshire ICB</t>
+  </si>
+  <si>
+    <t>E54000030</t>
+  </si>
+  <si>
+    <t>NHS South East London ICB</t>
   </si>
 </sst>
 </file>
@@ -194,7 +200,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7E41A41E-6BC1-4A66-967B-F05D38A218C0}" name="Table1" displayName="Table1" ref="A1:C15" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7E41A41E-6BC1-4A66-967B-F05D38A218C0}" name="Table1" displayName="Table1" ref="A1:C16" totalsRowShown="0">
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{8F2E8F24-AAEC-4353-A113-7527F65A6565}" name="nhs_region"/>
     <tableColumn id="2" xr3:uid="{00922057-391C-4CC6-A439-AC723AF49B76}" name="area_code"/>
@@ -467,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -510,13 +516,13 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -524,21 +530,21 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -546,21 +552,21 @@
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -568,21 +574,21 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -590,32 +596,32 @@
         <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -623,10 +629,10 @@
         <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -634,9 +640,20 @@
         <v>31</v>
       </c>
       <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
         <v>36</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C16" t="s">
         <v>37</v>
       </c>
     </row>

</xml_diff>